<commit_message>
store: 문의처를 admin@wellbian.io 로 정정
확정본의 admin@wellbianlab.io 는 사이트 도메인(wellbianlabs.io)과도 달라
확인을 요청했고, 서우가 wellbian.io 로 정정했다. 두 언어 모두 고쳤다.

영문은 주소 바로 뒤에 마침표가 오지 않게 문장을 바꿨다. 마침표를 주소의 일부로
집어삼키는 클라이언트가 있어서, 눌러도 열리지 않는 링크가 된다.

엑셀의 "결정 필요" 에서 도메인 항목을 내리고 "확정 사실" 로 옮겼다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014drgzQYBXTLjd1zzmsjRaS
</commit_message>
<xml_diff>
--- a/depin/content/faq-0830.xlsx
+++ b/depin/content/faq-0830.xlsx
@@ -836,7 +836,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>1계정당 최대 10대까지 신청하실 수 있습니다. 기업이나 대량 구매는 admin@wellbianlab.io 로 문의해 주세요.</t>
+          <t>1계정당 최대 10대까지 신청하실 수 있습니다. 기업이나 대량 구매는 admin@wellbian.io 로 문의해 주세요.</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Up to 10 per account. For business or bulk purchases, contact admin@wellbianlab.io.</t>
+          <t>Up to 10 per account. For business or bulk purchases, email admin@wellbian.io — we handle those separately.</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3164,22 +3164,22 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>문의 도메인 표기</t>
+          <t>기기 판매처</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>admin@wellbianlab.io</t>
+          <t>이 사이트 / KWeather 몰</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>사이트 도메인은 wellbianlabs.io(s 있음)인데 확정본 메일은 wellbianlab.io(s 없음)다. 둘 중 하나가 오타면 대량 구매 문의를 통째로 잃는다</t>
+          <t>옛 정본은 '기기는 KWeather 몰' 이라 했으나 사이트는 기기를 판다. 개정본에서는 뺐다</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>즉시</t>
+          <t>9/7 전</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
@@ -3189,51 +3189,51 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>기기 판매처</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>이 사이트 / KWeather 몰</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>옛 정본은 '기기는 KWeather 몰' 이라 했으나 사이트는 기기를 판다. 개정본에서는 뺐다</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>9/7 전</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>높음</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>2년 정확도 점검</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>근거 조항 미확인</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>미세먼지 특별법 조항을 찾아 약관에 넣기로 함. 확정되면 FAQ 문항 추가</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>9/15 전</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>중간</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>2년 정확도 점검</t>
+          <t>국내 거래소 지원 현황</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>근거 조항 미확인</t>
+          <t>코인원·디센트만 확인</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>미세먼지 특별법 조항을 찾아 약관에 넣기로 함. 확정되면 FAQ 문항 추가</t>
+          <t>b7 이 일반론으로 답한다. 거래소별 표를 줄 수 있으면 문의가 크게 준다</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>9/15 전</t>
+          <t>9/7 전</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -3245,22 +3245,22 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>국내 거래소 지원 현황</t>
+          <t>마이페이지 명칭</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>코인원·디센트만 확인</t>
+          <t>→ 데이터 보상</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>b7 이 일반론으로 답한다. 거래소별 표를 줄 수 있으면 문의가 크게 준다</t>
+          <t>회의 지시. 화면 문구와 FAQ 표현을 함께 바꿔야 한다</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>9/7 전</t>
+          <t>9/15 전</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -3272,17 +3272,17 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>마이페이지 명칭</t>
+          <t>보상 시작 시점</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>→ 데이터 보상</t>
+          <t>미정</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>회의 지시. 화면 문구와 FAQ 표현을 함께 바꿔야 한다</t>
+          <t>'언제부터 받나요' 가 자주 나올 텐데 b9 는 조건만 답한다</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -3299,17 +3299,17 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>보상 시작 시점</t>
+          <t>제네시스 부스트 배수</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>미정</t>
+          <t>미공개</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>'언제부터 받나요' 가 자주 나올 텐데 b9 는 조건만 답한다</t>
+          <t>x2 는 '보상 부스트' 라고만 쓴다. 수치를 낼지 결정</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -3319,78 +3319,78 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>중간</t>
+          <t>낮음</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>제네시스 부스트 배수</t>
+          <t>예매권 미수락 처리</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>미공개</t>
+          <t>미정</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>x2 는 '보상 부스트' 라고만 쓴다. 수치를 낼지 결정</t>
+          <t>마감까지 수락하지 않은 예매권을 어떻게 할지</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>9/15 전</t>
+          <t>9/14 전</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>낮음</t>
+          <t>중간</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>예매권 미수락 처리</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>미정</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>마감까지 수락하지 않은 예매권을 어떻게 할지</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>9/14 전</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>중간</t>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>지갑 키 보관 주체</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>미확인</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>자동 생성 지갑의 개인키를 누가 갖는지. 자산 관리 주체라 반드시 답이 있어야 하고, 답에 따라 문항 문안이 크게 달라진다</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>9/7 전</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>지갑 키 보관 주체</t>
+          <t>신청 후 수량 변경·취소</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>미정</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>자동 생성 지갑의 개인키를 누가 갖는지. 자산 관리 주체라 반드시 답이 있어야 하고, 답에 따라 문항 문안이 크게 달라진다</t>
+          <t>마감 전에 바꿀 수 있는지. 못 바꾸면 신청 화면에서 미리 알려야 한다</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
@@ -3405,81 +3405,54 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>신청 후 수량 변경·취소</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>미정</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>마감 전에 바꿀 수 있는지. 못 바꾸면 신청 화면에서 미리 알려야 한다</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>출금 수수료·소요 시간</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>거래소마다 상이</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>일반론만 답할 수 있다. 주요 거래소 기준값이 있으면 문의가 준다</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>9/7 전</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>높음</t>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>낮음</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>출금 수수료·소요 시간</t>
+          <t>실외·위성 기기 로드맵</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>거래소마다 상이</t>
+          <t>비공개</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>일반론만 답할 수 있다. 주요 거래소 기준값이 있으면 문의가 준다</t>
+          <t>TAXON 표에는 이미 있다. 물어보면 어디까지 답할지</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>9/7 전</t>
+          <t>미정</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>낮음</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>실외·위성 기기 로드맵</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>비공개</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>TAXON 표에는 이미 있다. 물어보면 어디까지 답할지</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>미정</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>낮음</t>
         </is>
@@ -3694,12 +3667,12 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>admin@wellbianlab.io</t>
+          <t>admin@wellbian.io</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>8/30 서우 확정 — 도메인 표기 확인 필요</t>
+          <t>8/30 서우 확정</t>
         </is>
       </c>
     </row>

</xml_diff>